<commit_message>
Actualizar el Excel con los arreglos del monitor moderno
Actualiza el inventario a 61 cambios e incorpora monitor físico, confinamiento del cursor, conservación de sesión, animaciones, garantía de renderers y suspensión de raycasts durante transiciones. Retira la descripción anterior del Canvas que ocupaba la cámara. Verificación: generador Node válido, rutas de implementación existentes, 61 entradas y partes XML del Excel bien formadas; resumen de 37 pruebas aprobadas y cero fallos.
</commit_message>
<xml_diff>
--- a/Docs/Cambios_Importantes_Archive_NULL.xlsx
+++ b/Docs/Cambios_Importantes_Archive_NULL.xlsx
@@ -105,7 +105,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" ht="64" customHeight="1">
@@ -128,7 +128,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">782d5de</t>
+          <t xml:space="preserve">75f97ff</t>
         </is>
       </c>
     </row>
@@ -152,7 +152,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">77 PASS y 0 FAIL en el último informe del editor.</t>
+          <t xml:space="preserve">37 PASS y 0 FAIL en el último informe del editor.</t>
         </is>
       </c>
     </row>
@@ -248,7 +248,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="64"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1681867</t>
+          <t xml:space="preserve">1e95557</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0e6a078</t>
+          <t xml:space="preserve">bb28fda</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0e6a078</t>
+          <t xml:space="preserve">bb28fda</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0e6a078</t>
+          <t xml:space="preserve">bb28fda</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La ejecución registrada midió 1,21 s de carga de recursos en regreso caliente; depende del equipo.</t>
+          <t xml:space="preserve">El tiempo del último regreso se registra como MEASURE en editor-mechanics.txt; depende del equipo y del estado de la caché.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1848,12 +1848,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vista sin recortes por escala del monitor</t>
+          <t xml:space="preserve">Escritorio dentro del monitor físico</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El Canvas principal independiente evita heredar la escala física del monitor.</t>
+          <t xml:space="preserve">Un Canvas de espacio de mundo se adapta a la superficie existente de la pantalla sin cubrir la cámara del jugador.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Captura del escritorio completo en la validación final.</t>
+          <t xml:space="preserve">Compilación y prueba del modo y anclaje del Canvas en editor.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1878,32 +1878,32 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expediente</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retratos de los cuatro personajes</t>
+          <t xml:space="preserve">Cursor limitado a la pantalla del ordenador</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El atlas proporciona retratos de Julián, Nicolás, Sofía y Víctor.</t>
+          <t xml:space="preserve">La posición del puntero se transforma a coordenadas de la pantalla física y se limita a sus bordes durante el foco.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CasePortraits.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/ModernOfficeDesktop.cs</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recurso de personajes ficticios y captura primary-case-file.png.</t>
+          <t xml:space="preserve">Pruebas de confinamiento y raycasts sobre botones del monitor.</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fd041c</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1913,32 +1913,32 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expediente</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reabrir información primaria desde el escritorio</t>
+          <t xml:space="preserve">Sesión visible al apartarse del ordenador</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El lector permite consultar el mismo expediente desde su carpeta y conserva proporciones de retratos.</t>
+          <t xml:space="preserve">Salir de la vista desactiva los clics y mantiene encendido el escritorio con la ventana que estaba abierta.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CaseFileReader.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/ModernOfficeDesktop.cs</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prueba de apertura desde Archive OS.</t>
+          <t xml:space="preserve">Prueba de conservación de ventana y liberación de raycasts.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1948,32 +1948,32 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leer el expediente antes de usar el ordenador</t>
+          <t xml:space="preserve">Animaciones de las ventanas</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sentarse y abrir el ordenador requieren descubrir la información primaria en la primera sesión.</t>
+          <t xml:space="preserve">Abrir, cerrar y minimizar combina fundido, escala y desplazamiento con curvas suavizadas; la barra restaura la ventana.</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/ModernOfficeDesktop.cs</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pruebas del bloqueo inicial y avance tras leer.</t>
+          <t xml:space="preserve">Pruebas de finalización de apertura, minimización, restauración y cierre.</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
     </row>
@@ -1983,32 +1983,32 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guía inicial de cinco pasos</t>
+          <t xml:space="preserve">Renderers de UI garantizados</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La ayuda conduce por expediente, asiento, escritorio, memoria y visor.</t>
+          <t xml:space="preserve">El controlador repara CanvasRenderer faltantes en Graphics serializados antes de aplicar el tema; los elementos nuevos lo crean explícitamente.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CRTMainMenuController.cs</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pruebas del flujo inicial; se oculta con otros paneles abiertos.</t>
+          <t xml:space="preserve">Compilación y comprobación de CanvasRenderer de todos los Graphics del escritorio.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">e025976</t>
         </is>
       </c>
     </row>
@@ -2018,32 +2018,32 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Memorias</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eliminar las dos pantallas de presentación</t>
+          <t xml:space="preserve">Suspender clics mientras se descarga la escena</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El inicio ya no instala las tarjetas antiguas de presentación.</t>
+          <t xml:space="preserve">La carga suspende raycasters del entorno saliente y restaura los que sobreviven al completar la transición.</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Narrative/DetectiveFantasyIntro.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/SceneFlow/MemoryLoadingScreen.cs</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Código y recorrido desde MainMenu.</t>
+          <t xml:space="preserve">37 comprobaciones aprobadas y cero fallos de runtime en la regresión del monitor; desaparece el error TitleText durante la descarga.</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4759ff1</t>
+          <t xml:space="preserve">bb28fda</t>
         </is>
       </c>
     </row>
@@ -2053,32 +2053,32 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Progresión</t>
+          <t xml:space="preserve">Expediente</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Requisitos claros para habilitar F1-Office</t>
+          <t xml:space="preserve">Retratos de los cuatro personajes</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La carpeta indica nota del estante, mensajes y llamadas; la huella sola no habilita la memoria.</t>
+          <t xml:space="preserve">El atlas proporciona retratos de Julián, Nicolás, Sofía y Víctor.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/CaseEvidenceCatalog.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CasePortraits.cs</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pruebas de requisitos y captura de carpetas.</t>
+          <t xml:space="preserve">Recurso de personajes ficticios y captura primary-case-file.png.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0108e41</t>
+          <t xml:space="preserve">0fd041c</t>
         </is>
       </c>
     </row>
@@ -2088,32 +2088,32 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Progresión</t>
+          <t xml:space="preserve">Expediente</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reparar desbloqueos de partidas anteriores</t>
+          <t xml:space="preserve">Reabrir información primaria desde el escritorio</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El índice de memorias se sincroniza con el desbloqueo guardado sin repetir el aviso.</t>
+          <t xml:space="preserve">El lector permite consultar el mismo expediente desde su carpeta y conserva proporciones de retratos.</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/EvidenceDrivenMemoryUnlock.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CaseFileReader.cs</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prueba de reparación de desbloqueo persistido.</t>
+          <t xml:space="preserve">Prueba de apertura desde Archive OS.</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0108e41</t>
+          <t xml:space="preserve">2037635</t>
         </is>
       </c>
     </row>
@@ -2123,32 +2123,32 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validación</t>
+          <t xml:space="preserve">Tutorial</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aislar partidas usadas en pruebas</t>
+          <t xml:space="preserve">Leer el expediente antes de usar el ordenador</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El argumento del editor fuerza guardados de laboratorio incluso al comenzar en la oficina.</t>
+          <t xml:space="preserve">Sentarse y abrir el ordenador requieren descubrir la información primaria en la primera sesión.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Core/GameSaveSystem.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Código y recorrido final con aislamiento.</t>
+          <t xml:space="preserve">Pruebas del bloqueo inicial y avance tras leer.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1681867</t>
+          <t xml:space="preserve">2037635</t>
         </is>
       </c>
     </row>
@@ -2158,32 +2158,32 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validación</t>
+          <t xml:space="preserve">Tutorial</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laboratorio de mecánicas en editor</t>
+          <t xml:space="preserve">Guía inicial de cinco pasos</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una escena permite probar colocación, fotografía, revelado y obstáculos.</t>
+          <t xml:space="preserve">La ayuda conduce por expediente, asiento, escritorio, memoria y visor.</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsLabEditor.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recorrido de laboratorio en Play Mode sin build de ejecutable.</t>
+          <t xml:space="preserve">Pruebas del flujo inicial; se oculta con otros paneles abiertos.</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">f1b4c99</t>
+          <t xml:space="preserve">2037635</t>
         </is>
       </c>
     </row>
@@ -2193,32 +2193,32 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validación</t>
+          <t xml:space="preserve">Tutorial</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recorrido automático ampliado</t>
+          <t xml:space="preserve">Eliminar las dos pantallas de presentación</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El probe recorre laboratorio, casa, oficina, escritorio, tutorial y herramientas.</t>
+          <t xml:space="preserve">El inicio ya no instala las tarjetas antiguas de presentación.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsEditorProbe.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Narrative/DetectiveFantasyIntro.cs</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">77 comprobaciones aprobadas y cero fallos en editor-mechanics.txt.</t>
+          <t xml:space="preserve">Código y recorrido desde MainMenu.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">f1b4c99</t>
+          <t xml:space="preserve">4759ff1</t>
         </is>
       </c>
     </row>
@@ -2228,37 +2228,212 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Progresión</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requisitos claros para habilitar F1-Office</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La carpeta indica nota del estante, mensajes y llamadas; la huella sola no habilita la memoria.</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/CaseEvidenceCatalog.cs</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pruebas de requisitos y captura de carpetas.</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0108e41</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="64" customHeight="1">
+      <c r="A58" s="2">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Progresión</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reparar desbloqueos de partidas anteriores</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El índice de memorias se sincroniza con el desbloqueo guardado sin repetir el aviso.</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/EvidenceDrivenMemoryUnlock.cs</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prueba de reparación de desbloqueo persistido.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0108e41</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="64" customHeight="1">
+      <c r="A59" s="3">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Validación</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aislar partidas usadas en pruebas</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El argumento del editor fuerza guardados de laboratorio incluso al comenzar en la oficina.</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Core/GameSaveSystem.cs</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Código y recorrido final con aislamiento.</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e95557</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="64" customHeight="1">
+      <c r="A60" s="2">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validación</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laboratorio de mecánicas en editor</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Una escena permite probar colocación, fotografía, revelado y obstáculos.</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsLabEditor.cs</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recorrido de laboratorio en Play Mode sin build de ejecutable.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e95557</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="64" customHeight="1">
+      <c r="A61" s="3">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validación</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recorrido automático ampliado</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El probe permite el recorrido completo o la validación específica del monitor, tutorial, progresión y herramientas de oficina.</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsEditorProbe.cs</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado del último recorrido en la hoja Resumen y en editor-mechanics.txt; el alcance depende del modo ejecutado.</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e95557</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="64" customHeight="1">
+      <c r="A62" s="2">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validación</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Prueba de oficina independiente</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">El comando OfficeOnly inicia el recorrido del editor en MainMenu.</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tools/Test-EditorMechanics.ps1</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Revisión del argumento y entrada de editor; guardados aislados.</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">f1b4c99</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G57"/>
+  <autoFilter ref="A1:G62"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9"/>
 </worksheet>
@@ -2294,204 +2469,205 @@
     <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">782d5de</t>
+          <t xml:space="preserve">75f97ff</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar los resultados y capturas de la validación en editor</t>
+          <t xml:space="preserve">Documentar y registrar la regresión limpia del monitor físico</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actualiza el informe de 77 comprobaciones aprobadas y las capturas del juego. Añade imágenes de Archive OS, carpetas y expediente. El regreso con recursos de oficina conservados midió 1,21 segundos en esta ejecución; no garantiza el mismo tiempo en todos los equipos.</t>
+          <t xml:space="preserve">Actualiza la guía del monitor en la escena, cursor limitado, sesión persistente y animaciones. Registra el recorrido final con 37 comprobaciones aprobadas y cero fallos de runtime, junto con capturas del escritorio físico, expediente y oficina. La carga caliente de regreso midió 1,23 segundos en esta ejecución. Verificación: informe final y revisión visual de la barra de tareas dentro del marco; preferencias del usuario restauradas.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">372edb3</t>
+          <t xml:space="preserve">bb28fda</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actualizar la guía de escritorio, progresión y herramientas</t>
+          <t xml:space="preserve">Evitar raycasts sobre renderers que se descargan durante la carga</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documenta el tutorial inicial, las carpetas de Archive OS, los retratos, los requisitos de F1-Office y las herramientas permitidas en F1-House. Explica la corrección de colocación. Verificación: contraste con las implementaciones y el recorrido final del editor.</t>
+          <t xml:space="preserve">Suspende los raycasters activos de la escena saliente mientras cambia el entorno y restaura únicamente los que sobreviven al terminar. Elimina la excepción CanvasRenderer de TitleText que se reprodujo durante la salida de la oficina. La primera ejecución del recorrido tuvo 37 comprobaciones de comportamiento aprobadas pero errores de runtime, por lo que la descripción previa de la prueba no bastaba para acreditar un recorrido limpio. Verificación final: 37 comprobaciones aprobadas y cero errores de runtime en el viaje oficina–F1-Office–oficina; escritorio y barra revisados en captura física del monitor.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="100" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">f1b4c99</t>
+          <t xml:space="preserve">2111d69</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ampliar las pruebas en editor para escritorio, tutorial y colocación</t>
+          <t xml:space="preserve">Ajustar el escritorio al área visible del marco del monitor</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Añade comprobaciones de Archive OS, lectura obligatoria, desbloqueo, restricciones de herramientas y colocación en ambas memorias. Permite ejecutar solamente la oficina desde PowerShell. Verificación previa de la tanda completa: 77 comprobaciones aprobadas y ningún fallo; no se generó un ejecutable.</t>
+          <t xml:space="preserve">Reduce la altura útil de la superficie conservando su borde superior para que la barra de tareas no quede detrás del plástico inferior. Expone el ajuste de altura en el controlador. Verificación: compilación sin errores y comparación de la captura del monitor; la captura actualizada se revisa en la siguiente ejecución.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="100" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1681867</t>
+          <t xml:space="preserve">1e95557</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aislar los guardados de las pruebas automáticas del editor</t>
+          <t xml:space="preserve">Verificar el monitor físico en la sesión abierta del editor</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El argumento de pruebas activa el directorio de guardados del laboratorio incluso cuando el recorrido comienza en MainMenu. Evita que la prueba de oficina use los guardados de juego del usuario. Verificación: recorrido final en editor con el argumento de aislamiento.</t>
+          <t xml:space="preserve">Añade un recorrido de oficina en el editor abierto sin regenerar el laboratorio, con guardados aislados. Comprueba anclaje en el monitor, raycasts de botones, confinamiento del cursor, CanvasRenderer, conservación de sesión y animaciones de apertura, minimización, restauración y cierre. Verificación: recorrido de oficina completado sin fallos, incluyendo regreso desde F1-Office. No se generó un ejecutable.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">605436d</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reemplazar el menú CRT por un escritorio moderno interactivo</t>
+          <t xml:space="preserve">Animar apertura, cierre y minimización de ventanas del escritorio</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Introduce Archive OS con arranque, aplicaciones, carpetas, ventanas movibles y minimizables, barra de tareas y selección de memorias. Conserva las referencias serializadas del controlador anterior. Integra expediente, informe y configuración; corrige el cursor al cerrar opciones y evita que la escala del monitor recorte el escritorio. Verificación: arranque, navegación, expediente, opciones y montaje de memoria en Play Mode; capturas de escritorio y carpetas.</t>
+          <t xml:space="preserve">Añade fundidos, desplazamiento breve y escala suavizada con tiempo independiente de la pausa. Bloquea los botones mientras la ventana transiciona y restaura ventanas minimizadas desde la barra de tareas. Verificación: compilación de scripts sin errores; se añade comprobación de transición y restauración al recorrido de editor.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="100" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">e025976</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guiar el inicio y exigir la lectura del expediente antes de sentarse</t>
+          <t xml:space="preserve">Integrar Archive OS en la pantalla física del monitor</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Añade una guía persistente por pasos y bloquea el acceso al asiento y ordenador hasta abrir la información primaria. Sincroniza el tutorial hablado con esa lectura. El expediente muestra retratos conservando proporciones, mejora su fuente y permite reapertura desde el escritorio. Verificación: bloqueo inicial, apertura del expediente y avance del tutorial en la prueba final de Play Mode.</t>
+          <t xml:space="preserve">Reemplaza el Canvas de pantalla completa por un Canvas en espacio de mundo ajustado a la superficie existente. Limita el cursor al monitor y convierte el arrastre a coordenadas locales de esa pantalla. Al salir conserva la ventana visible y libera la interacción; al cargar una memoria apaga el monitor. Verificación: compilación de todos los scripts sin errores; las pruebas de raycast y foco se incorporan en la regresión del editor.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="100" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0108e41</t>
+          <t xml:space="preserve">c5f7054</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reparar el desbloqueo persistente de la segunda memoria</t>
+          <t xml:space="preserve">Garantizar CanvasRenderer en los textos del monitor</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sincroniza el índice de archivos con el desbloqueo guardado de F1-Office. Expone una actualización de progreso y un listado de requisitos: nota del estante, mensajes y llamadas. Evita repetir el aviso si la memoria ya estaba habilitada. Verificación: pruebas finales de requisitos y reparación de preferencias antiguas.</t>
+          <t xml:space="preserve">Repara los Graphics serializados antes de aplicar el tema del monitor y crea los elementos nuevos con CanvasRenderer explícito. Adelanta la inicialización del controlador para evitar acceso de TMP a componentes faltantes. Verificación: compilación de los scripts de Unity sin errores; la regresión en Play Mode se realiza con los siguientes ajustes del monitor.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0713ec0</t>
+          <t xml:space="preserve">98491c6</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corregir la colocación de herramientas y su disponibilidad en la casa</t>
+          <t xml:space="preserve">Documentar 56 cambios importantes del juego en un Excel verificable</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Excluye los colliders del operador de los rayos y comprueba penetración real para evitar falsos obstáculos en mallas grandes. Corrige colocación, recogida de tags y apuntado al trípode. Oculta trípode y linterna blanca en F1-House y bloquea sus atajos; conserva UV. Verificación: pruebas finales de colocación y recogida en casa y oficina, y restricciones de la rueda.</t>
+          <t xml:space="preserve">Incluye hojas de resumen, cambios y commits con descripciones en español, rutas existentes, alcance de validación y referencias reales de Git. Distingue el último commit de cada archivo del origen histórico de cada comportamiento.
+Añade un generador OOXML sin dependencias externas para mantener el inventario. Verificación: sintaxis de Node, exportación correcta, XML bien formado y 56 identificadores únicos. Registra las 77 comprobaciones aprobadas del editor sin afirmar nuevas pruebas del juego ni generar ejecutables.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="100" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4759ff1</t>
+          <t xml:space="preserve">782d5de</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retirar las dos presentaciones iniciales</t>
+          <t xml:space="preserve">Registrar los resultados y capturas de la validación en editor</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elimina las tarjetas de presentación y su instalación automática. Mantiene un componente compatible con las referencias serializadas que elimina cualquier instancia antigua. Verificación: recorrido de inicio en MainMenu dentro de la prueba final de Play Mode.</t>
+          <t xml:space="preserve">Actualiza el informe de 77 comprobaciones aprobadas y las capturas del juego. Añade imágenes de Archive OS, carpetas y expediente. El regreso con recursos de oficina conservados midió 1,21 segundos en esta ejecución; no garantiza el mismo tiempo en todos los equipos.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="100" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fd041c</t>
+          <t xml:space="preserve">372edb3</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Añadir retratos de los personajes del expediente</t>
+          <t xml:space="preserve">Actualizar la guía de escritorio, progresión y herramientas</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incorpora un atlas de cuatro personajes ficticios y su proveedor de sprites. Conserva las proporciones del recurso y sus metadatos de Unity. La integración con el lector se realiza en el cambio del tutorial. Verificación: recurso presente y retratos usados por la prueba final del expediente en Play Mode.</t>
+          <t xml:space="preserve">Documenta el tutorial inicial, las carpetas de Archive OS, los retratos, los requisitos de F1-Office y las herramientas permitidas en F1-House. Explica la corrección de colocación. Verificación: contraste con las implementaciones y el recorrido final del editor.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="100" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">56145cb</t>
+          <t xml:space="preserve">f1b4c99</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Excluir preferencias locales y resultados temporales de pruebas</t>
+          <t xml:space="preserve">Ampliar las pruebas en editor para escritorio, tutorial y colocación</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retira del seguimiento la copia del registro de PlayerPrefs y conserva el archivo local. Ignora esa copia y el resultado temporal de diagnóstico de la casa. Verificación: rutas específicas en .gitignore; no se modifica el historial previo.</t>
+          <t xml:space="preserve">Añade comprobaciones de Archive OS, lectura obligatoria, desbloqueo, restricciones de herramientas y colocación en ambas memorias. Permite ejecutar solamente la oficina desde PowerShell. Verificación previa de la tanda completa: 77 comprobaciones aprobadas y ningún fallo; no se generó un ejecutable.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="100" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9232e94</t>
+          <t xml:space="preserve">1681867</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentar commits atómicos en español y validación en editor</t>
+          <t xml:space="preserve">Aislar los guardados de las pruebas automáticas del editor</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registra las preferencias del usuario para separar cambios coherentes, describir su propósito y revisar cada diff. Mantiene la validación en editor y el inventario de cambios del juego. Verificación: lectura de las reglas del proyecto.</t>
+          <t xml:space="preserve">El argumento de pruebas activa el directorio de guardados del laboratorio incluso cuando el recorrido comienza en MainMenu. Evita que la prueba de oficina use los guardados de juego del usuario. Verificación: recorrido final en editor con el argumento de aislamiento.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar el Excel con 70 mejoras verificables del juego
Añade nueve mejoras de la oficina: opciones en el monitor, cursor y sonidos propios, eliminación de pausa en MainMenu, altura estable, llegada a la puerta, regreso sentado y movimiento con pasos de alfombra. Regenera las tres hojas con rutas, referencias de commits y el resultado de editor de 55 PASS y 0 FAIL. Verificados sintaxis del generador, estructura XML del XLSX y 70 identificadores únicos.
</commit_message>
<xml_diff>
--- a/Docs/Cambios_Importantes_Archive_NULL.xlsx
+++ b/Docs/Cambios_Importantes_Archive_NULL.xlsx
@@ -105,7 +105,7 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" ht="64" customHeight="1">
@@ -128,7 +128,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">75f97ff</t>
+          <t xml:space="preserve">459fa29</t>
         </is>
       </c>
     </row>
@@ -152,7 +152,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">37 PASS y 0 FAIL en el último informe del editor.</t>
+          <t xml:space="preserve">55 PASS y 0 FAIL en el último informe del editor.</t>
         </is>
       </c>
     </row>
@@ -248,7 +248,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr defaultRowHeight="64"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e95557</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb28fda</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb28fda</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb28fda</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">54425ab</t>
+          <t xml:space="preserve">6965f6f</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">a81a8ca</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
     </row>
@@ -2038,12 +2038,12 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">37 comprobaciones aprobadas y cero fallos de runtime en la regresión del monitor; desaparece el error TitleText durante la descarga.</t>
+          <t xml:space="preserve">Conteo del recorrido vigente en la hoja Resumen; consultas a renderers descargados suspendidas durante el cambio de escena.</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb28fda</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
     </row>
@@ -2053,32 +2053,32 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expediente</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retratos de los cuatro personajes</t>
+          <t xml:space="preserve">Retirar la interacción del CRT anterior</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El atlas proporciona retratos de Julián, Nicolás, Sofía y Víctor.</t>
+          <t xml:space="preserve">El Canvas del monitor anterior deja de recibir raycasts y sus textos dejan de ser objetivos del puntero.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CasePortraits.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CRTMainMenuController.Desktop.cs</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recurso de personajes ficticios y captura primary-case-file.png.</t>
+          <t xml:space="preserve">Compilación y regresión de apertura, opciones y cambio de escena sin el raycaster del CRT.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fd041c</t>
+          <t xml:space="preserve">a81a8ca</t>
         </is>
       </c>
     </row>
@@ -2088,32 +2088,32 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expediente</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reabrir información primaria desde el escritorio</t>
+          <t xml:space="preserve">Ajustes dentro de la pantalla física</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El lector permite consultar el mismo expediente desde su carpeta y conserva proporciones de retratos.</t>
+          <t xml:space="preserve">General, Sonido, Video, Idioma y Controles aparecen como pestañas de una ventana del ordenador.</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CaseFileReader.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/ModernOfficeDesktop.Settings.cs</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prueba de apertura desde Archive OS.</t>
+          <t xml:space="preserve">Pruebas de paneles, sliders y persistencia de intensidad corporal en el monitor.</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">6965f6f</t>
         </is>
       </c>
     </row>
@@ -2123,32 +2123,32 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leer el expediente antes de usar el ordenador</t>
+          <t xml:space="preserve">Oficina sin menú de pausa</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sentarse y abrir el ordenador requieren descubrir la información primaria en la primera sesión.</t>
+          <t xml:space="preserve">Las entradas públicas a pausa y configuración no crean un overlay ni detienen MainMenu.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Menu/Pausa/GlobalPauseMenu.cs</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pruebas del bloqueo inicial y avance tras leer.</t>
+          <t xml:space="preserve">Pruebas de ausencia de instancia de pausa y tiempo continuo al configurar en oficina.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">6965f6f</t>
         </is>
       </c>
     </row>
@@ -2158,32 +2158,32 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guía inicial de cinco pasos</t>
+          <t xml:space="preserve">Cursor propio de Archive OS</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">La ayuda conduce por expediente, asiento, escritorio, memoria y visor.</t>
+          <t xml:space="preserve">Un gráfico del juego sustituye al puntero del sistema y se mantiene completo dentro de los bordes del monitor.</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/ModernOfficeDesktop.Feedback.cs</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pruebas del flujo inicial; se oculta con otros paneles abiertos.</t>
+          <t xml:space="preserve">Pruebas de cursor propio, puntero del sistema oculto y superficie física del escritorio.</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2037635</t>
+          <t xml:space="preserve">00ea7a2</t>
         </is>
       </c>
     </row>
@@ -2193,32 +2193,32 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutorial</t>
+          <t xml:space="preserve">Escritorio</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eliminar las dos pantallas de presentación</t>
+          <t xml:space="preserve">Sonidos del ordenador</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El inicio ya no instala las tarjetas antiguas de presentación.</t>
+          <t xml:space="preserve">Inicio, apertura, cierre, clic y hover tienen sonidos breves que respetan el volumen de efectos.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Narrative/DetectiveFantasyIntro.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/ModernOfficeDesktop.Feedback.cs</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Código y recorrido desde MainMenu.</t>
+          <t xml:space="preserve">Compilación y prueba de inicialización de audio; timbre generado evaluable en Play Mode.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4759ff1</t>
+          <t xml:space="preserve">00ea7a2</t>
         </is>
       </c>
     </row>
@@ -2228,32 +2228,32 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Progresión</t>
+          <t xml:space="preserve">Oficina</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Requisitos claros para habilitar F1-Office</t>
+          <t xml:space="preserve">Altura estable al levantarse</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">La carpeta indica nota del estante, mensajes y llamadas; la huella sola no habilita la memoria.</t>
+          <t xml:space="preserve">La vista al estar de pie conserva la altura de llegada y evita capturar alturas intermedias al salir del asiento.</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/CaseEvidenceCatalog.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CRTMenuCameraFocus.cs</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pruebas de requisitos y captura de carpetas.</t>
+          <t xml:space="preserve">Prueba de altura después de levantarse del escritorio.</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0108e41</t>
+          <t xml:space="preserve">a81a8ca</t>
         </is>
       </c>
     </row>
@@ -2263,32 +2263,32 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Progresión</t>
+          <t xml:space="preserve">Oficina</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reparar desbloqueos de partidas anteriores</t>
+          <t xml:space="preserve">Llegada a la puerta en cada sesión nueva</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">El índice de memorias se sincroniza con el desbloqueo guardado sin repetir el aviso.</t>
+          <t xml:space="preserve">Un inicio de juego aparece en el spawn de la puerta independientemente del avance del tutorial o una posición guardada.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/EvidenceDrivenMemoryUnlock.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CRTMenuCameraFocus.cs</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prueba de reparación de desbloqueo persistido.</t>
+          <t xml:space="preserve">Pruebas de spawn inicial y elección de pose con tutorial completado.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0108e41</t>
+          <t xml:space="preserve">a81a8ca</t>
         </is>
       </c>
     </row>
@@ -2298,32 +2298,32 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validación</t>
+          <t xml:space="preserve">Oficina</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aislar partidas usadas en pruebas</t>
+          <t xml:space="preserve">Regreso sentado desde memoria</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El argumento del editor fuerza guardados de laboratorio incluso al comenzar en la oficina.</t>
+          <t xml:space="preserve">La transición activa identifica el regreso y coloca al jugador sentado ante el escritorio.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Core/GameSaveSystem.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/SceneFlow/MemoryLoadingScreen.cs</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Código y recorrido final con aislamiento.</t>
+          <t xml:space="preserve">Prueba de posición sentada tras oficina–F1-Office–oficina.</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e95557</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
     </row>
@@ -2333,32 +2333,32 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validación</t>
+          <t xml:space="preserve">Oficina</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laboratorio de mecánicas en editor</t>
+          <t xml:space="preserve">Movimiento corporal y pasos de alfombra</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una escena permite probar colocación, fotografía, revelado y obstáculos.</t>
+          <t xml:space="preserve">El controlador propio incorpora balanceo y respiración, con pasos amortiguados según distancia recorrida.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsLabEditor.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeFreeLookController.Feedback.cs</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recorrido de laboratorio en Play Mode sin build de ejecutable.</t>
+          <t xml:space="preserve">Entrada real en Play Mode activa balanceo y pasos; altura estable comprobada. Timbre y sensación corporal evaluables por el jugador.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e95557</t>
+          <t xml:space="preserve">16e87f8</t>
         </is>
       </c>
     </row>
@@ -2368,32 +2368,32 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validación</t>
+          <t xml:space="preserve">Expediente</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recorrido automático ampliado</t>
+          <t xml:space="preserve">Retratos de los cuatro personajes</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El probe permite el recorrido completo o la validación específica del monitor, tutorial, progresión y herramientas de oficina.</t>
+          <t xml:space="preserve">El atlas proporciona retratos de Julián, Nicolás, Sofía y Víctor.</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsEditorProbe.cs</t>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CasePortraits.cs</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resultado del último recorrido en la hoja Resumen y en editor-mechanics.txt; el alcance depende del modo ejecutado.</t>
+          <t xml:space="preserve">Recurso de personajes ficticios y captura primary-case-file.png.</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e95557</t>
+          <t xml:space="preserve">0fd041c</t>
         </is>
       </c>
     </row>
@@ -2403,37 +2403,352 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Expediente</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reabrir información primaria desde el escritorio</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El lector permite consultar el mismo expediente desde su carpeta y conserva proporciones de retratos.</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/CaseFileReader.cs</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prueba de apertura desde Archive OS.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2037635</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="64" customHeight="1">
+      <c r="A63" s="3">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tutorial</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leer el expediente antes de usar el ordenador</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sentarse y abrir el ordenador requieren descubrir la información primaria en la primera sesión.</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pruebas del bloqueo inicial y avance tras leer.</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2037635</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="64" customHeight="1">
+      <c r="A64" s="2">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tutorial</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guía inicial de cinco pasos</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La ayuda conduce por expediente, asiento, escritorio, memoria y visor.</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Office/OfficeOnboarding.cs</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pruebas del flujo inicial; se oculta con otros paneles abiertos.</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2037635</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="64" customHeight="1">
+      <c r="A65" s="3">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tutorial</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eliminar las dos pantallas de presentación</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El inicio ya no instala las tarjetas antiguas de presentación.</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Narrative/DetectiveFantasyIntro.cs</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Código y recorrido desde MainMenu.</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4759ff1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="64" customHeight="1">
+      <c r="A66" s="2">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Progresión</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requisitos claros para habilitar F1-Office</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La carpeta indica nota del estante, mensajes y llamadas; la huella sola no habilita la memoria.</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/CaseEvidenceCatalog.cs</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pruebas de requisitos y captura de carpetas.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0108e41</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="64" customHeight="1">
+      <c r="A67" s="3">
+        <v>66</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Progresión</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reparar desbloqueos de partidas anteriores</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El índice de memorias se sincroniza con el desbloqueo guardado sin repetir el aviso.</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Evidence/EvidenceDrivenMemoryUnlock.cs</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prueba de reparación de desbloqueo persistido.</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0108e41</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="64" customHeight="1">
+      <c r="A68" s="2">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Validación</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aislar partidas usadas en pruebas</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El argumento del editor fuerza guardados de laboratorio incluso al comenzar en la oficina.</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Scripts/Core/GameSaveSystem.cs</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Código y recorrido final con aislamiento.</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f119edf</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="64" customHeight="1">
+      <c r="A69" s="3">
+        <v>68</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validación</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laboratorio de mecánicas en editor</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Una escena permite probar colocación, fotografía, revelado y obstáculos.</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsLabEditor.cs</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recorrido de laboratorio en Play Mode sin build de ejecutable.</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e95557</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="64" customHeight="1">
+      <c r="A70" s="2">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validación</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recorrido automático ampliado</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El probe permite el recorrido completo o la validación específica del monitor, tutorial, progresión y herramientas de oficina.</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assets/ArchiveNull/Editor/MechanicsEditorProbe.cs</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado del último recorrido en la hoja Resumen y en editor-mechanics.txt; el alcance depende del modo ejecutado.</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1ada2fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="64" customHeight="1">
+      <c r="A71" s="3">
+        <v>70</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validación</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Prueba de oficina independiente</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">El comando OfficeOnly inicia el recorrido del editor en MainMenu.</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E71" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tools/Test-EditorMechanics.ps1</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F71" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Revisión del argumento y entrada de editor; guardados aislados.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">f1b4c99</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G62"/>
+  <autoFilter ref="A1:G71"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9"/>
 </worksheet>
@@ -2469,205 +2784,204 @@
     <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">75f97ff</t>
+          <t xml:space="preserve">459fa29</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentar y registrar la regresión limpia del monitor físico</t>
+          <t xml:space="preserve">Documentar los ajustes del monitor y la regresión de oficina</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actualiza la guía del monitor en la escena, cursor limitado, sesión persistente y animaciones. Registra el recorrido final con 37 comprobaciones aprobadas y cero fallos de runtime, junto con capturas del escritorio físico, expediente y oficina. La carga caliente de regreso midió 1,23 segundos en esta ejecución. Verificación: informe final y revisión visual de la barra de tareas dentro del marco; preferencias del usuario restauradas.</t>
+          <t xml:space="preserve">Actualiza la guía de Play Mode con el cursor propio, sonidos, ajustes físicos del ordenador y reglas de llegada y regreso. Conserva resultados y capturas del recorrido oficina–F1-Office–oficina: 55 PASS, 0 FAIL, con movimiento real y retorno sentado comprobados.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb28fda</t>
+          <t xml:space="preserve">1ada2fc</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evitar raycasts sobre renderers que se descargan durante la carga</t>
+          <t xml:space="preserve">Verificar movimiento y ajustes de la oficina en Play Mode</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suspende los raycasters activos de la escena saliente mientras cambia el entorno y restaura únicamente los que sobreviven al terminar. Elimina la excepción CanvasRenderer de TitleText que se reprodujo durante la salida de la oficina. La primera ejecución del recorrido tuvo 37 comprobaciones de comportamiento aprobadas pero errores de runtime, por lo que la descripción previa de la prueba no bastaba para acreditar un recorrido limpio. Verificación final: 37 comprobaciones aprobadas y cero errores de runtime en el viaje oficina–F1-Office–oficina; escritorio y barra revisados en captura física del monitor.</t>
+          <t xml:space="preserve">Amplía la regresión con llegada a la puerta, altura al levantarse, desplazamiento mediante entrada real, pasos de alfombra, cursor propio y opciones dentro del monitor. Comprueba también el regreso sentado desde F1-Office y que MainMenu no cree pausa. Validación en el editor: 55 comprobaciones aprobadas y cero fallos; sin build del juego.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="100" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111d69</t>
+          <t xml:space="preserve">40e4807</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ajustar el escritorio al área visible del marco del monitor</t>
+          <t xml:space="preserve">Mantener completo el cursor propio dentro de los bordes del monitor</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reduce la altura útil de la superficie conservando su borde superior para que la barra de tareas no quede detrás del plástico inferior. Expone el ajuste de altura en el controlador. Verificación: compilación sin errores y comparación de la captura del monitor; la captura actualizada se revisa en la siguiente ejecución.</t>
+          <t xml:space="preserve">Reserva espacio para el ancho y alto del cursor dibujado al confinar el puntero. Evita que casi todo el gráfico quede recortado por la máscara al alcanzar los bordes derecho e inferior. Verificación: compilación sin errores; se comprueba la visibilidad del puntero en la regresión del monitor.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="100" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e95557</t>
+          <t xml:space="preserve">a81a8ca</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificar el monitor físico en la sesión abierta del editor</t>
+          <t xml:space="preserve">Proteger la reasignación de teclas frente a la salida del escritorio</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Añade un recorrido de oficina en el editor abierto sin regenerar el laboratorio, con guardados aislados. Comprueba anclaje en el monitor, raycasts de botones, confinamiento del cursor, CanvasRenderer, conservación de sesión y animaciones de apertura, minimización, restauración y cierre. Verificación: recorrido de oficina completado sin fallos, incluyendo regreso desde F1-Office. No se generó un ejecutable.</t>
+          <t xml:space="preserve">Consulta la reasignación activa a través del controlador del monitor, aunque el componente de foco esté en otro objeto. Evita que Escape cierre el escritorio mientras se cancela una nueva tecla. Verificación: compilación de scripts sin errores y pestaña Controles disponible dentro del monitor.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">605436d</t>
+          <t xml:space="preserve">b1f7092</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Animar apertura, cierre y minimización de ventanas del escritorio</t>
+          <t xml:space="preserve">Conservar la altura de llegada también durante el desplazamiento libre</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Añade fundidos, desplazamiento breve y escala suavizada con tiempo independiente de la pausa. Bloquea los botones mientras la ventana transiciona y restaura ventanas minimizadas desde la barra de tareas. Verificación: compilación de scripts sin errores; se añade comprobación de transición y restauración al recorrido de editor.</t>
+          <t xml:space="preserve">El movimiento horizontal consulta la altura de pie del controlador de poses para evitar usar una altura capturada antes de que termine su inicialización. Verificación: compilación sin errores y prueba de altura tras levantarse aprobada en el recorrido de oficina.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="100" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">e025976</t>
+          <t xml:space="preserve">16e87f8</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrar Archive OS en la pantalla física del monitor</t>
+          <t xml:space="preserve">Añadir movimiento corporal y pasos de alfombra en la oficina</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reemplaza el Canvas de pantalla completa por un Canvas en espacio de mundo ajustado a la superficie existente. Limita el cursor al monitor y convierte el arrastre a coordenadas locales de esa pantalla. Al salir conserva la ventana visible y libera la interacción; al cargar una memoria apaga el monitor. Verificación: compilación de todos los scripts sin errores; las pruebas de raycast y foco se incorporan en la regresión del editor.</t>
+          <t xml:space="preserve">Integra pasos, balanceo corporal y respiración en el controlador propio de MainMenu sin aplicar el controlador de las memorias. Usa la distancia realmente recorrida para los sonidos amortiguados de alfombra y elimina el desplazamiento visual antes de la siguiente actualización para no alterar altura ni colisiones. Comparte sensibilidad y teclas del ordenador. Verificación: compilación sin errores; el recorrido del editor comprueba altura estable y disponibilidad de sonidos al caminar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="100" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">c5f7054</t>
+          <t xml:space="preserve">00ea7a2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Garantizar CanvasRenderer en los textos del monitor</t>
+          <t xml:space="preserve">Añadir cursor propio y sonidos de interacción al ordenador</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repara los Graphics serializados antes de aplicar el tema del monitor y crea los elementos nuevos con CanvasRenderer explícito. Adelanta la inicialización del controlador para evitar acceso de TMP a componentes faltantes. Verificación: compilación de los scripts de Unity sin errores; la regresión en Play Mode se realiza con los siguientes ajustes del monitor.</t>
+          <t xml:space="preserve">Dibuja un puntero de Archive OS dentro del monitor y oculta el cursor del sistema durante su uso. Añade sonidos breves de inicio, apertura, cierre, clic y hover con volumen de efectos compartido. Libera los recursos generados al descargar la escena. Verificación: compilación de scripts sin errores; se añaden comprobaciones de cursor, fuente de audio y configuración integrada al recorrido de oficina.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="100" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">98491c6</t>
+          <t xml:space="preserve">f119edf</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentar 56 cambios importantes del juego en un Excel verificable</t>
+          <t xml:space="preserve">Conservar altura al levantarse y distinguir llegada de regreso a memoria</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incluye hojas de resumen, cambios y commits con descripciones en español, rutas existentes, alcance de validación y referencias reales de Git. Distingue el último commit de cada archivo del origen histórico de cada comportamiento.
-Añade un generador OOXML sin dependencias externas para mantener el inventario. Verificación: sintaxis de Node, exportación correcta, XML bien formado y 56 identificadores únicos. Registra las 77 comprobaciones aprobadas del editor sin afirmar nuevas pruebas del juego ni generar ejecutables.</t>
+          <t xml:space="preserve">Usa la llegada desde MemoryLoadingScreen para volver sentado y reserva el spawn de la puerta para cada inicio de sesión, sin depender del tutorial ni de una preferencia de reconstrucción. Conserva la altura inicial al levantarse y evita que el movimiento libre capture una altura intermedia durante la transición. No restaura la posición guardada de MainMenu. Verificación: compilación sin errores; se añaden comprobaciones de altura, puerta y regreso sentado al recorrido de oficina.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="100" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">782d5de</t>
+          <t xml:space="preserve">6965f6f</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar los resultados y capturas de la validación en editor</t>
+          <t xml:space="preserve">Integrar todos los ajustes en una ventana del ordenador de la oficina</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actualiza el informe de 77 comprobaciones aprobadas y las capturas del juego. Añade imágenes de Archive OS, carpetas y expediente. El regreso con recursos de oficina conservados midió 1,21 segundos en esta ejecución; no garantiza el mismo tiempo en todos los equipos.</t>
+          <t xml:space="preserve">Sustituye las opciones superpuestas por pestañas General, Sonido, Video, Idioma y Controles dentro del monitor físico, con valores persistentes y reasignación de teclas. Impide crear o pausar GlobalPauseMenu en MainMenu, incluso desde llamadas públicas. Verificación: compilación sin errores; se amplía la regresión para comprobar que la configuración no pausa ni crea un overlay.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="100" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">372edb3</t>
+          <t xml:space="preserve">1ac7872</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actualizar la guía de escritorio, progresión y herramientas</t>
+          <t xml:space="preserve">Retirar los raycasts y textos interactivos del monitor CRT anterior</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documenta el tutorial inicial, las carpetas de Archive OS, los retratos, los requisitos de F1-Office y las herramientas permitidas en F1-House. Explica la corrección de colocación. Verificación: contraste con las implementaciones y el recorrido final del editor.</t>
+          <t xml:space="preserve">Desactiva permanentemente el GraphicRaycaster del Canvas antiguo y deja sus textos fuera de las consultas de puntero. Solo el escritorio moderno recibe clics del monitor; evita que el EventSystem consulte TitleText retirados junto a la nueva interfaz. Verificación: compilación de scripts sin errores; el caso de regresión de apertura, configuración y cambio de escena se verifica en editor al completar la tanda.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="100" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">f1b4c99</t>
+          <t xml:space="preserve">4b6994b</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ampliar las pruebas en editor para escritorio, tutorial y colocación</t>
+          <t xml:space="preserve">Actualizar el Excel con los arreglos del monitor moderno</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Añade comprobaciones de Archive OS, lectura obligatoria, desbloqueo, restricciones de herramientas y colocación en ambas memorias. Permite ejecutar solamente la oficina desde PowerShell. Verificación previa de la tanda completa: 77 comprobaciones aprobadas y ningún fallo; no se generó un ejecutable.</t>
+          <t xml:space="preserve">Actualiza el inventario a 61 cambios e incorpora monitor físico, confinamiento del cursor, conservación de sesión, animaciones, garantía de renderers y suspensión de raycasts durante transiciones. Retira la descripción anterior del Canvas que ocupaba la cámara. Verificación: generador Node válido, rutas de implementación existentes, 61 entradas y partes XML del Excel bien formadas; resumen de 37 pruebas aprobadas y cero fallos.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="100" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1681867</t>
+          <t xml:space="preserve">75f97ff</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aislar los guardados de las pruebas automáticas del editor</t>
+          <t xml:space="preserve">Documentar y registrar la regresión limpia del monitor físico</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">El argumento de pruebas activa el directorio de guardados del laboratorio incluso cuando el recorrido comienza en MainMenu. Evita que la prueba de oficina use los guardados de juego del usuario. Verificación: recorrido final en editor con el argumento de aislamiento.</t>
+          <t xml:space="preserve">Actualiza la guía del monitor en la escena, cursor limitado, sesión persistente y animaciones. Registra el recorrido final con 37 comprobaciones aprobadas y cero fallos de runtime, junto con capturas del escritorio físico, expediente y oficina. La carga caliente de regreso midió 1,23 segundos en esta ejecución. Verificación: informe final y revisión visual de la barra de tareas dentro del marco; preferencias del usuario restauradas.</t>
         </is>
       </c>
     </row>

</xml_diff>